<commit_message>
Agregar limpieza de cod_local (6 dígitos), cod_mod (7 dígitos, sep /) y actualizar do-file
- cod_local: pad con ceros a la izquierda hasta 6 dígitos, letras = missing
- cod_mod: cada código padded a 7 dígitos, múltiples separados por /,
  letras y texto descriptivo = missing
- CUI: solo numérico (sin cambios)
- do-file: reescrito completo con código corregido del usuario +
  secciones nuevas de cod_local y cod_mod
- Detección automática de entorno Windows/Linux para rutas

https://claude.ai/code/session_01UxQcKqmPzHwUBumpNBSpJS
</commit_message>
<xml_diff>
--- a/Anexo1_base_errores.xlsx
+++ b/Anexo1_base_errores.xlsx
@@ -642,7 +642,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>20606</t>
+          <t>020606</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -705,11 +705,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>SE INTERVENDRAN EN: COCINA</t>
-        </is>
-      </c>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
           <t>NO</t>
@@ -821,7 +817,7 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20606</t>
+          <t>020606</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -884,11 +880,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>INSTALACIONES DEPORTIVAS</t>
-        </is>
-      </c>
+      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1000,7 +992,7 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>20606</t>
+          <t>020606</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1063,11 +1055,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>LOSA DEPORTIVA</t>
-        </is>
-      </c>
+      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1179,7 +1167,7 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>20606</t>
+          <t>020606</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1242,11 +1230,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>LOSA DEPORTIVA</t>
-        </is>
-      </c>
+      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1362,7 +1346,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>20625</t>
+          <t>020625</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1425,11 +1409,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>-----------------------</t>
-        </is>
-      </c>
+      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1608,11 +1588,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>-----------------------</t>
-        </is>
-      </c>
+      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1728,7 +1704,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>34335</t>
+          <t>034335</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1859,7 +1835,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>16015</t>
+          <t>016015</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1994,7 +1970,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>24807</t>
+          <t>024807</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2236,11 +2212,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
           <t>NO</t>
@@ -2419,11 +2391,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
           <t>NO</t>
@@ -2539,7 +2507,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>21371</t>
+          <t>021371</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2817,7 +2785,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>45230</t>
+          <t>045230</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2992,7 +2960,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>47521</t>
+          <t>047521</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3119,7 +3087,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>47540</t>
+          <t>047540</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -3290,7 +3258,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>47559</t>
+          <t>047559</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -3417,7 +3385,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>47564</t>
+          <t>047564</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3544,7 +3512,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>47583</t>
+          <t>047583</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3715,7 +3683,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>47601</t>
+          <t>047601</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -3886,7 +3854,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>47615</t>
+          <t>047615</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -4013,7 +3981,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>47658</t>
+          <t>047658</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -4136,7 +4104,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>47663</t>
+          <t>047663</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -4942,7 +4910,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>79814</t>
+          <t>079814</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -5121,7 +5089,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>80011</t>
+          <t>080011</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -5300,7 +5268,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>89196</t>
+          <t>089196</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -5365,7 +5333,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>89196</t>
+          <t>0089196</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -5910,7 +5878,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>438259</t>
+          <t>0438259</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -6089,7 +6057,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>438648</t>
+          <t>0438648</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
@@ -6443,7 +6411,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>391128</t>
+          <t>0391128</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
@@ -6622,7 +6590,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>390732</t>
+          <t>0390732</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
@@ -8094,11 +8062,7 @@
       </c>
       <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr">
         <is>
           <t>NO</t>
@@ -9781,7 +9745,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>206086</t>
+          <t>0206086</t>
         </is>
       </c>
       <c r="P60" t="inlineStr">
@@ -10143,7 +10107,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>207449</t>
+          <t>0207449</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
@@ -10503,11 +10467,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O64" t="inlineStr">
-        <is>
-          <t>_</t>
-        </is>
-      </c>
+      <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr">
         <is>
           <t>&lt;&lt;ERROR&gt;&gt;</t>
@@ -10686,11 +10646,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O65" t="inlineStr">
-        <is>
-          <t>_</t>
-        </is>
-      </c>
+      <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr">
         <is>
           <t>&lt;&lt;ERROR&gt;&gt;</t>
@@ -10869,11 +10825,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O66" t="inlineStr">
-        <is>
-          <t>_</t>
-        </is>
-      </c>
+      <c r="O66" t="inlineStr"/>
       <c r="P66" t="inlineStr">
         <is>
           <t>&lt;&lt;ERROR&gt;&gt;</t>
@@ -11052,11 +11004,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O67" t="inlineStr">
-        <is>
-          <t>_</t>
-        </is>
-      </c>
+      <c r="O67" t="inlineStr"/>
       <c r="P67" t="inlineStr">
         <is>
           <t>&lt;&lt;ERROR&gt;&gt;</t>
@@ -11172,7 +11120,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>47045</t>
+          <t>047045</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -13025,11 +12973,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="O78" t="inlineStr">
-        <is>
-          <t>NINGUNA</t>
-        </is>
-      </c>
+      <c r="O78" t="inlineStr"/>
       <c r="P78" t="inlineStr">
         <is>
           <t>SI</t>
@@ -13208,11 +13152,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="O79" t="inlineStr">
-        <is>
-          <t>NINGUNA</t>
-        </is>
-      </c>
+      <c r="O79" t="inlineStr"/>
       <c r="P79" t="inlineStr">
         <is>
           <t>SI</t>
@@ -13391,11 +13331,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="O80" t="inlineStr">
-        <is>
-          <t>NINGUNA</t>
-        </is>
-      </c>
+      <c r="O80" t="inlineStr"/>
       <c r="P80" t="inlineStr">
         <is>
           <t>SI</t>
@@ -13988,7 +13924,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>52640</t>
+          <t>052640</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -14051,11 +13987,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="O84" t="inlineStr">
-        <is>
-          <t>I.E.I. 475-5</t>
-        </is>
-      </c>
+      <c r="O84" t="inlineStr"/>
       <c r="P84" t="inlineStr">
         <is>
           <t>SI</t>
@@ -14230,11 +14162,7 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="O85" t="inlineStr">
-        <is>
-          <t>ALFONSO RODRIGUEZ NAJARRO</t>
-        </is>
-      </c>
+      <c r="O85" t="inlineStr"/>
       <c r="P85" t="inlineStr">
         <is>
           <t>NO</t>
@@ -15045,11 +14973,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O90" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="O90" t="inlineStr"/>
       <c r="P90" t="inlineStr">
         <is>
           <t>NO</t>
@@ -15220,11 +15144,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O91" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="O91" t="inlineStr"/>
       <c r="P91" t="inlineStr">
         <is>
           <t>NO</t>
@@ -15395,11 +15315,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O92" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="O92" t="inlineStr"/>
       <c r="P92" t="inlineStr"/>
       <c r="Q92" t="inlineStr"/>
       <c r="R92" t="inlineStr"/>
@@ -15534,11 +15450,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O93" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="O93" t="inlineStr"/>
       <c r="P93" t="inlineStr">
         <is>
           <t>NO</t>
@@ -15709,11 +15621,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O94" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="O94" t="inlineStr"/>
       <c r="P94" t="inlineStr">
         <is>
           <t>NO</t>
@@ -15884,11 +15792,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O95" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="O95" t="inlineStr"/>
       <c r="P95" t="inlineStr">
         <is>
           <t>NO</t>
@@ -16063,11 +15967,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O96" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O96" t="inlineStr"/>
       <c r="P96" t="inlineStr">
         <is>
           <t>SI</t>
@@ -16234,11 +16134,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O97" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O97" t="inlineStr"/>
       <c r="P97" t="inlineStr">
         <is>
           <t>SI</t>
@@ -16405,11 +16301,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O98" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O98" t="inlineStr"/>
       <c r="P98" t="inlineStr">
         <is>
           <t>SI</t>
@@ -16580,11 +16472,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O99" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O99" t="inlineStr"/>
       <c r="P99" t="inlineStr">
         <is>
           <t>SI</t>
@@ -16751,11 +16639,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O100" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O100" t="inlineStr"/>
       <c r="P100" t="inlineStr">
         <is>
           <t>SI</t>
@@ -16922,11 +16806,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O101" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O101" t="inlineStr"/>
       <c r="P101" t="inlineStr">
         <is>
           <t>SI</t>
@@ -17093,11 +16973,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O102" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O102" t="inlineStr"/>
       <c r="P102" t="inlineStr">
         <is>
           <t>SI</t>
@@ -17264,11 +17140,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O103" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O103" t="inlineStr"/>
       <c r="P103" t="inlineStr">
         <is>
           <t>SI</t>
@@ -17435,11 +17307,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O104" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O104" t="inlineStr"/>
       <c r="P104" t="inlineStr">
         <is>
           <t>SI</t>
@@ -17610,11 +17478,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O105" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O105" t="inlineStr"/>
       <c r="P105" t="inlineStr">
         <is>
           <t>SI</t>
@@ -17785,11 +17649,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O106" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O106" t="inlineStr"/>
       <c r="P106" t="inlineStr">
         <is>
           <t>SI</t>
@@ -17960,11 +17820,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O107" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O107" t="inlineStr"/>
       <c r="P107" t="inlineStr">
         <is>
           <t>SI</t>
@@ -18135,11 +17991,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O108" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O108" t="inlineStr"/>
       <c r="P108" t="inlineStr">
         <is>
           <t>SI</t>
@@ -18310,11 +18162,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O109" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O109" t="inlineStr"/>
       <c r="P109" t="inlineStr">
         <is>
           <t>SI</t>
@@ -18485,11 +18333,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O110" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O110" t="inlineStr"/>
       <c r="P110" t="inlineStr">
         <is>
           <t>SI</t>
@@ -18656,11 +18500,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O111" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O111" t="inlineStr"/>
       <c r="P111" t="inlineStr">
         <is>
           <t>SI</t>
@@ -18827,11 +18667,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O112" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O112" t="inlineStr"/>
       <c r="P112" t="inlineStr">
         <is>
           <t>SI</t>
@@ -18998,11 +18834,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O113" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O113" t="inlineStr"/>
       <c r="P113" t="inlineStr">
         <is>
           <t>SI</t>
@@ -19169,11 +19001,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O114" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O114" t="inlineStr"/>
       <c r="P114" t="inlineStr">
         <is>
           <t>SI</t>
@@ -19340,11 +19168,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O115" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O115" t="inlineStr"/>
       <c r="P115" t="inlineStr">
         <is>
           <t>SI</t>
@@ -19511,11 +19335,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O116" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O116" t="inlineStr"/>
       <c r="P116" t="inlineStr">
         <is>
           <t>SI</t>
@@ -19682,11 +19502,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O117" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O117" t="inlineStr"/>
       <c r="P117" t="inlineStr">
         <is>
           <t>SI</t>
@@ -19853,11 +19669,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O118" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O118" t="inlineStr"/>
       <c r="P118" t="inlineStr">
         <is>
           <t>SI</t>
@@ -20028,11 +19840,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O119" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O119" t="inlineStr"/>
       <c r="P119" t="inlineStr">
         <is>
           <t>SI</t>
@@ -20203,11 +20011,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O120" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O120" t="inlineStr"/>
       <c r="P120" t="inlineStr">
         <is>
           <t>SI</t>
@@ -20378,11 +20182,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O121" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O121" t="inlineStr"/>
       <c r="P121" t="inlineStr">
         <is>
           <t>SI</t>
@@ -20553,11 +20353,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O122" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O122" t="inlineStr"/>
       <c r="P122" t="inlineStr">
         <is>
           <t>SI</t>
@@ -20728,11 +20524,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O123" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O123" t="inlineStr"/>
       <c r="P123" t="inlineStr">
         <is>
           <t>SI</t>
@@ -20903,11 +20695,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O124" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O124" t="inlineStr"/>
       <c r="P124" t="inlineStr">
         <is>
           <t>SI</t>
@@ -21078,11 +20866,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O125" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O125" t="inlineStr"/>
       <c r="P125" t="inlineStr">
         <is>
           <t>SI</t>
@@ -21253,11 +21037,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O126" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="O126" t="inlineStr"/>
       <c r="P126" t="inlineStr">
         <is>
           <t>SI</t>
@@ -21428,11 +21208,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="O127" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="O127" t="inlineStr"/>
       <c r="P127" t="inlineStr">
         <is>
           <t>SI</t>
@@ -21607,11 +21383,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O128" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="O128" t="inlineStr"/>
       <c r="P128" t="inlineStr">
         <is>
           <t>&lt;&lt;ERROR&gt;&gt;</t>
@@ -26271,11 +26043,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O156" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="O156" t="inlineStr"/>
       <c r="P156" t="inlineStr">
         <is>
           <t>&lt;&lt;ERROR&gt;&gt;</t>
@@ -26450,11 +26218,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O157" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="O157" t="inlineStr"/>
       <c r="P157" t="inlineStr">
         <is>
           <t>&lt;&lt;ERROR&gt;&gt;</t>
@@ -26629,11 +26393,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O158" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="O158" t="inlineStr"/>
       <c r="P158" t="inlineStr">
         <is>
           <t>&lt;&lt;ERROR&gt;&gt;</t>
@@ -26808,11 +26568,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O159" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="O159" t="inlineStr"/>
       <c r="P159" t="inlineStr">
         <is>
           <t>&lt;&lt;ERROR&gt;&gt;</t>
@@ -26987,11 +26743,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O160" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="O160" t="inlineStr"/>
       <c r="P160" t="inlineStr">
         <is>
           <t>&lt;&lt;ERROR&gt;&gt;</t>
@@ -27166,11 +26918,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O161" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="O161" t="inlineStr"/>
       <c r="P161" t="inlineStr">
         <is>
           <t>&lt;&lt;ERROR&gt;&gt;</t>
@@ -27345,11 +27093,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O162" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="O162" t="inlineStr"/>
       <c r="P162" t="inlineStr">
         <is>
           <t>&lt;&lt;ERROR&gt;&gt;</t>
@@ -27524,11 +27268,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O163" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="O163" t="inlineStr"/>
       <c r="P163" t="inlineStr">
         <is>
           <t>&lt;&lt;ERROR&gt;&gt;</t>
@@ -27703,11 +27443,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O164" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="O164" t="inlineStr"/>
       <c r="P164" t="inlineStr">
         <is>
           <t>&lt;&lt;ERROR&gt;&gt;</t>
@@ -27882,11 +27618,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="O165" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="O165" t="inlineStr"/>
       <c r="P165" t="inlineStr">
         <is>
           <t>NO</t>
@@ -28057,11 +27789,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O166" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="O166" t="inlineStr"/>
       <c r="P166" t="inlineStr">
         <is>
           <t>&lt;&lt;ERROR&gt;&gt;</t>
@@ -28232,11 +27960,7 @@
         </is>
       </c>
       <c r="N167" t="inlineStr"/>
-      <c r="O167" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="O167" t="inlineStr"/>
       <c r="P167" t="inlineStr">
         <is>
           <t>SI</t>
@@ -28407,11 +28131,7 @@
         </is>
       </c>
       <c r="N168" t="inlineStr"/>
-      <c r="O168" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="O168" t="inlineStr"/>
       <c r="P168" t="inlineStr">
         <is>
           <t>SI</t>
@@ -28578,11 +28298,7 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="O169" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="O169" t="inlineStr"/>
       <c r="P169" t="inlineStr">
         <is>
           <t>NO</t>
@@ -28757,11 +28473,7 @@
           <t>&lt;&lt;ERROR&gt;&gt;</t>
         </is>
       </c>
-      <c r="O170" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="O170" t="inlineStr"/>
       <c r="P170" t="inlineStr">
         <is>
           <t>&lt;&lt;ERROR&gt;&gt;</t>
@@ -29117,7 +28829,7 @@
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>321067</t>
+          <t>0321067</t>
         </is>
       </c>
       <c r="P172" t="inlineStr">

</xml_diff>